<commit_message>
cambios en outline, pptx, en script principal es que se añadieron los nutrientes de Bombuscaro
</commit_message>
<xml_diff>
--- a/NUMEX_pre_RStudio/data_for_R.xlsx
+++ b/NUMEX_pre_RStudio/data_for_R.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC181"/>
+  <dimension ref="A1:BB181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -690,15 +690,10 @@
       </c>
       <c r="BA1" s="1" t="inlineStr">
         <is>
-          <t>Carea</t>
+          <t>N</t>
         </is>
       </c>
       <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
@@ -845,15 +840,12 @@
         <v>-1.069204566063425</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.1583411527786951</v>
+        <v>1.583411527786951</v>
       </c>
       <c r="BA2" t="n">
-        <v>6.267862957094129</v>
+        <v>0</v>
       </c>
       <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -998,15 +990,12 @@
         <v>-1.162714378482783</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0.1927929018543231</v>
+        <v>1.927929018543231</v>
       </c>
       <c r="BA3" t="n">
-        <v>4.931398966307422</v>
+        <v>1</v>
       </c>
       <c r="BB3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1151,15 +1140,12 @@
         <v>-1.083217188451016</v>
       </c>
       <c r="AZ4" t="n">
-        <v>0.1459443363957555</v>
+        <v>1.459443363957554</v>
       </c>
       <c r="BA4" t="n">
-        <v>6.201410491775166</v>
+        <v>0</v>
       </c>
       <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1304,15 +1290,12 @@
         <v>-1.173469655199274</v>
       </c>
       <c r="AZ5" t="n">
-        <v>0.2308390026071944</v>
+        <v>2.308390026071943</v>
       </c>
       <c r="BA5" t="n">
-        <v>6.803966990152447</v>
+        <v>1</v>
       </c>
       <c r="BB5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1457,15 +1440,12 @@
         <v>-1.152717050430573</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.1972952651382424</v>
+        <v>1.972952651382424</v>
       </c>
       <c r="BA6" t="n">
-        <v>5.814010355624786</v>
+        <v>1</v>
       </c>
       <c r="BB6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1610,15 +1590,12 @@
         <v>-0.9757692279498354</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0.2411024955423218</v>
+        <v>2.411024955423218</v>
       </c>
       <c r="BA7" t="n">
-        <v>6.393667365779264</v>
+        <v>0</v>
       </c>
       <c r="BB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1763,15 +1740,12 @@
         <v>-1.066817746219274</v>
       </c>
       <c r="AZ8" t="n">
-        <v>0.2212734935521185</v>
+        <v>2.212734935521185</v>
       </c>
       <c r="BA8" t="n">
-        <v>6.582919875238116</v>
+        <v>0</v>
       </c>
       <c r="BB8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1916,15 +1890,12 @@
         <v>-1.120257664680253</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.2491330280495736</v>
+        <v>2.491330280495736</v>
       </c>
       <c r="BA9" t="n">
-        <v>7.04653963916366</v>
+        <v>0</v>
       </c>
       <c r="BB9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2069,15 +2040,12 @@
         <v>-1.176763154946914</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.1922442143630735</v>
+        <v>1.922442143630735</v>
       </c>
       <c r="BA10" t="n">
-        <v>5.385976820401974</v>
+        <v>0</v>
       </c>
       <c r="BB10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2222,15 +2190,12 @@
         <v>-1.083133704760353</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.1541538771183675</v>
+        <v>1.541538771183675</v>
       </c>
       <c r="BA11" t="n">
-        <v>6.156964889603419</v>
+        <v>1</v>
       </c>
       <c r="BB11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2375,15 +2340,12 @@
         <v>-0.9693632665794485</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.1704503359635594</v>
+        <v>1.704503359635594</v>
       </c>
       <c r="BA12" t="n">
-        <v>7.04539122144526</v>
+        <v>1</v>
       </c>
       <c r="BB12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2528,15 +2490,12 @@
         <v>-1.01178671221848</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.1893086604314295</v>
+        <v>1.893086604314296</v>
       </c>
       <c r="BA13" t="n">
-        <v>6.298227944361334</v>
+        <v>0</v>
       </c>
       <c r="BB13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2681,15 +2640,12 @@
         <v>-0.9086318732906992</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.2420263723581012</v>
+        <v>2.420263723581012</v>
       </c>
       <c r="BA14" t="n">
-        <v>5.933547349313596</v>
+        <v>0</v>
       </c>
       <c r="BB14" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2834,15 +2790,12 @@
         <v>-0.9710658232898745</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.2262696828216982</v>
+        <v>2.262696828216981</v>
       </c>
       <c r="BA15" t="n">
-        <v>6.737742901484933</v>
+        <v>1</v>
       </c>
       <c r="BB15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2987,15 +2940,12 @@
         <v>-1.011623867625123</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.2346594974817987</v>
+        <v>2.346594974817986</v>
       </c>
       <c r="BA16" t="n">
-        <v>7.585479688556592</v>
+        <v>1</v>
       </c>
       <c r="BB16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3140,15 +3090,12 @@
         <v>-1.137930339273472</v>
       </c>
       <c r="AZ17" t="n">
-        <v>0.2040293659175826</v>
+        <v>2.040293659175827</v>
       </c>
       <c r="BA17" t="n">
-        <v>5.793309073325802</v>
+        <v>1</v>
       </c>
       <c r="BB17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3293,15 +3240,12 @@
         <v>-0.9983195512068304</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0.2199748552043699</v>
+        <v>2.199748552043698</v>
       </c>
       <c r="BA18" t="n">
-        <v>6.418104834646514</v>
+        <v>0</v>
       </c>
       <c r="BB18" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3446,15 +3390,12 @@
         <v>-1.159881181147376</v>
       </c>
       <c r="AZ19" t="n">
-        <v>0.1804095984933663</v>
+        <v>1.804095984933663</v>
       </c>
       <c r="BA19" t="n">
-        <v>4.811120672929789</v>
+        <v>0</v>
       </c>
       <c r="BB19" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3599,15 +3540,12 @@
         <v>-1.14385783446787</v>
       </c>
       <c r="AZ20" t="n">
-        <v>0.2216436966512492</v>
+        <v>2.216436966512492</v>
       </c>
       <c r="BA20" t="n">
-        <v>6.816510648324604</v>
+        <v>1</v>
       </c>
       <c r="BB20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3752,15 +3690,12 @@
         <v>-0.8250529055541557</v>
       </c>
       <c r="AZ21" t="n">
-        <v>0.2731252805030631</v>
+        <v>2.731252805030631</v>
       </c>
       <c r="BA21" t="n">
-        <v>6.269341168086865</v>
+        <v>1</v>
       </c>
       <c r="BB21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3905,15 +3840,12 @@
         <v>-0.9307778716019919</v>
       </c>
       <c r="AZ22" t="n">
-        <v>0.1359691165823957</v>
+        <v>1.359691165823957</v>
       </c>
       <c r="BA22" t="n">
-        <v>7.209869586996444</v>
+        <v>0</v>
       </c>
       <c r="BB22" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4058,15 +3990,12 @@
         <v>-1.076624094600751</v>
       </c>
       <c r="AZ23" t="n">
-        <v>0.1532285064088778</v>
+        <v>1.532285064088778</v>
       </c>
       <c r="BA23" t="n">
-        <v>5.8814772925756</v>
+        <v>0</v>
       </c>
       <c r="BB23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4211,15 +4140,12 @@
         <v>-0.9531215121310557</v>
       </c>
       <c r="AZ24" t="n">
-        <v>0.2083919474390169</v>
+        <v>2.083919474390169</v>
       </c>
       <c r="BA24" t="n">
-        <v>6.450269324889292</v>
+        <v>0</v>
       </c>
       <c r="BB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4364,15 +4290,12 @@
         <v>-1.127672428671739</v>
       </c>
       <c r="AZ25" t="n">
-        <v>0.1924962019984864</v>
+        <v>1.924962019984864</v>
       </c>
       <c r="BA25" t="n">
-        <v>5.922628309595306</v>
+        <v>1</v>
       </c>
       <c r="BB25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC25" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4517,15 +4440,12 @@
         <v>-1.093730835683608</v>
       </c>
       <c r="AZ26" t="n">
-        <v>0.1993680458705612</v>
+        <v>1.993680458705612</v>
       </c>
       <c r="BA26" t="n">
-        <v>5.819873982352418</v>
+        <v>1</v>
       </c>
       <c r="BB26" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4670,15 +4590,12 @@
         <v>-0.9251981278059437</v>
       </c>
       <c r="AZ27" t="n">
-        <v>0.2247906864753312</v>
+        <v>2.247906864753312</v>
       </c>
       <c r="BA27" t="n">
-        <v>4.353630630525455</v>
+        <v>1</v>
       </c>
       <c r="BB27" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4823,15 +4740,12 @@
         <v>-1.110646754176239</v>
       </c>
       <c r="AZ28" t="n">
-        <v>0.1941969337398241</v>
+        <v>1.941969337398241</v>
       </c>
       <c r="BA28" t="n">
-        <v>6.180318961158282</v>
+        <v>0</v>
       </c>
       <c r="BB28" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4976,15 +4890,12 @@
         <v>-0.8721981465115956</v>
       </c>
       <c r="AZ29" t="n">
-        <v>0.2299853817964811</v>
+        <v>2.299853817964811</v>
       </c>
       <c r="BA29" t="n">
-        <v>4.77039521233669</v>
+        <v>0</v>
       </c>
       <c r="BB29" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5129,15 +5040,12 @@
         <v>-1.026018023099852</v>
       </c>
       <c r="AZ30" t="n">
-        <v>0.2056480718564838</v>
+        <v>2.056480718564837</v>
       </c>
       <c r="BA30" t="n">
-        <v>6.003256549989229</v>
+        <v>0</v>
       </c>
       <c r="BB30" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5282,15 +5190,12 @@
         <v>-1.081725628636109</v>
       </c>
       <c r="AZ31" t="n">
-        <v>0.136631885562437</v>
+        <v>1.36631885562437</v>
       </c>
       <c r="BA31" t="n">
-        <v>5.871422404388254</v>
+        <v>0</v>
       </c>
       <c r="BB31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5435,15 +5340,12 @@
         <v>-0.9757257325131097</v>
       </c>
       <c r="AZ32" t="n">
-        <v>0.2060536274187499</v>
+        <v>2.060536274187499</v>
       </c>
       <c r="BA32" t="n">
-        <v>4.248872527334292</v>
+        <v>0</v>
       </c>
       <c r="BB32" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC32" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5588,15 +5490,12 @@
         <v>-1.108000186694067</v>
       </c>
       <c r="AZ33" t="n">
-        <v>0.2140487849336566</v>
+        <v>2.140487849336566</v>
       </c>
       <c r="BA33" t="n">
-        <v>4.707179999838402</v>
+        <v>0</v>
       </c>
       <c r="BB33" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5741,15 +5640,12 @@
         <v>-1.1317622997201</v>
       </c>
       <c r="AZ34" t="n">
-        <v>0.1262484116656832</v>
+        <v>1.262484116656831</v>
       </c>
       <c r="BA34" t="n">
-        <v>5.538752547725021</v>
+        <v>0</v>
       </c>
       <c r="BB34" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5894,15 +5790,12 @@
         <v>-1.097985206987246</v>
       </c>
       <c r="AZ35" t="n">
-        <v>0.236853606683806</v>
+        <v>2.36853606683806</v>
       </c>
       <c r="BA35" t="n">
-        <v>5.72708070874746</v>
+        <v>0</v>
       </c>
       <c r="BB35" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC35" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6047,15 +5940,12 @@
         <v>-1.041003254864917</v>
       </c>
       <c r="AZ36" t="n">
-        <v>0.1404492354378129</v>
+        <v>1.404492354378129</v>
       </c>
       <c r="BA36" t="n">
-        <v>6.421580057406096</v>
+        <v>0</v>
       </c>
       <c r="BB36" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC36" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6200,15 +6090,12 @@
         <v>-1.128326182974303</v>
       </c>
       <c r="AZ37" t="n">
-        <v>0.165736668134432</v>
+        <v>1.65736668134432</v>
       </c>
       <c r="BA37" t="n">
-        <v>5.382476778431748</v>
+        <v>1</v>
       </c>
       <c r="BB37" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6353,15 +6240,12 @@
         <v>-1.052221717593601</v>
       </c>
       <c r="AZ38" t="n">
-        <v>0.25370946862891</v>
+        <v>2.5370946862891</v>
       </c>
       <c r="BA38" t="n">
-        <v>7.926449640071605</v>
+        <v>1</v>
       </c>
       <c r="BB38" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6506,15 +6390,12 @@
         <v>-1.018263130425242</v>
       </c>
       <c r="AZ39" t="n">
-        <v>0.1790085898974969</v>
+        <v>1.790085898974969</v>
       </c>
       <c r="BA39" t="n">
-        <v>3.990234824028318</v>
+        <v>1</v>
       </c>
       <c r="BB39" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6659,15 +6540,12 @@
         <v>-1.134852638614013</v>
       </c>
       <c r="AZ40" t="n">
-        <v>0.1636334848571583</v>
+        <v>1.636334848571583</v>
       </c>
       <c r="BA40" t="n">
-        <v>6.701960533465813</v>
+        <v>1</v>
       </c>
       <c r="BB40" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC40" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6812,15 +6690,12 @@
         <v>-1.046794083447492</v>
       </c>
       <c r="AZ41" t="n">
-        <v>0.1962293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BA41" t="n">
-        <v>6.406993482654983</v>
+        <v>0</v>
       </c>
       <c r="BB41" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6965,15 +6840,12 @@
         <v>-1.055363556422817</v>
       </c>
       <c r="AZ42" t="n">
-        <v>0.1962293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BA42" t="n">
-        <v>6.406993482654983</v>
+        <v>0</v>
       </c>
       <c r="BB42" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7118,15 +6990,12 @@
         <v>-1.027478472194354</v>
       </c>
       <c r="AZ43" t="n">
-        <v>0.1962293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BA43" t="n">
-        <v>6.406993482654983</v>
+        <v>0</v>
       </c>
       <c r="BB43" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7271,15 +7140,12 @@
         <v>-1.035889819888641</v>
       </c>
       <c r="AZ44" t="n">
-        <v>0.1962293560349081</v>
+        <v>1.962293560349081</v>
       </c>
       <c r="BA44" t="n">
-        <v>6.406993482654983</v>
+        <v>0</v>
       </c>
       <c r="BB44" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC44" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7424,15 +7290,12 @@
         <v>-1.016944806660762</v>
       </c>
       <c r="AZ45" t="n">
-        <v>0.2080347916779913</v>
+        <v>2.080347916779913</v>
       </c>
       <c r="BA45" t="n">
-        <v>7.270477607848516</v>
+        <v>0</v>
       </c>
       <c r="BB45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7577,15 +7440,12 @@
         <v>-1.168428613749502</v>
       </c>
       <c r="AZ46" t="n">
-        <v>0.1803572361821152</v>
+        <v>1.803572361821152</v>
       </c>
       <c r="BA46" t="n">
-        <v>4.981358951370535</v>
+        <v>0</v>
       </c>
       <c r="BB46" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7730,15 +7590,12 @@
         <v>-1.006406074511895</v>
       </c>
       <c r="AZ47" t="n">
-        <v>0.1563233988308393</v>
+        <v>1.563233988308393</v>
       </c>
       <c r="BA47" t="n">
-        <v>4.941560931653564</v>
+        <v>0</v>
       </c>
       <c r="BB47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7883,15 +7740,12 @@
         <v>-1.002974473340656</v>
       </c>
       <c r="AZ48" t="n">
-        <v>0.1727182447385554</v>
+        <v>1.727182447385554</v>
       </c>
       <c r="BA48" t="n">
-        <v>5.627608137299266</v>
+        <v>0</v>
       </c>
       <c r="BB48" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8036,15 +7890,12 @@
         <v>-1.033343565098957</v>
       </c>
       <c r="AZ49" t="n">
-        <v>0.2118768969038876</v>
+        <v>2.118768969038876</v>
       </c>
       <c r="BA49" t="n">
-        <v>7.860992204916545</v>
+        <v>1</v>
       </c>
       <c r="BB49" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8189,15 +8040,12 @@
         <v>-1.094831536193773</v>
       </c>
       <c r="AZ50" t="n">
-        <v>0.1305405133948935</v>
+        <v>1.305405133948935</v>
       </c>
       <c r="BA50" t="n">
-        <v>6.085878779925097</v>
+        <v>1</v>
       </c>
       <c r="BB50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8342,15 +8190,12 @@
         <v>-1.034130614924995</v>
       </c>
       <c r="AZ51" t="n">
-        <v>0.2749705279828398</v>
+        <v>2.749705279828397</v>
       </c>
       <c r="BA51" t="n">
-        <v>7.600880368696366</v>
+        <v>1</v>
       </c>
       <c r="BB51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8495,15 +8340,12 @@
         <v>-0.9330413776996519</v>
       </c>
       <c r="AZ52" t="n">
-        <v>0.2554237568151246</v>
+        <v>2.554237568151246</v>
       </c>
       <c r="BA52" t="n">
-        <v>8.029662939995131</v>
+        <v>1</v>
       </c>
       <c r="BB52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8645,12 +8487,9 @@
       </c>
       <c r="AZ53" t="inlineStr"/>
       <c r="BA53" t="n">
-        <v>3.469168210591955</v>
+        <v>1</v>
       </c>
       <c r="BB53" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC53" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8795,15 +8634,12 @@
         <v>-1.09799079624996</v>
       </c>
       <c r="AZ54" t="n">
-        <v>0.2230482700063978</v>
+        <v>2.230482700063977</v>
       </c>
       <c r="BA54" t="n">
-        <v>3.834114387266885</v>
+        <v>1</v>
       </c>
       <c r="BB54" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC54" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8948,15 +8784,12 @@
         <v>-1.013558134662488</v>
       </c>
       <c r="AZ55" t="n">
-        <v>0.2700331914670088</v>
+        <v>2.700331914670088</v>
       </c>
       <c r="BA55" t="n">
-        <v>9.226808188432537</v>
+        <v>0</v>
       </c>
       <c r="BB55" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC55" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9101,15 +8934,12 @@
         <v>-1.029758709416929</v>
       </c>
       <c r="AZ56" t="n">
-        <v>0.1811914954031918</v>
+        <v>1.811914954031917</v>
       </c>
       <c r="BA56" t="n">
-        <v>5.640759522824799</v>
+        <v>0</v>
       </c>
       <c r="BB56" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC56" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9254,15 +9084,12 @@
         <v>-1.071407723597514</v>
       </c>
       <c r="AZ57" t="n">
-        <v>0.1485071659290358</v>
+        <v>1.485071659290358</v>
       </c>
       <c r="BA57" t="n">
-        <v>6.279270830799232</v>
+        <v>0</v>
       </c>
       <c r="BB57" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9407,15 +9234,12 @@
         <v>-1.076020463092165</v>
       </c>
       <c r="AZ58" t="n">
-        <v>0.181805467668072</v>
+        <v>1.818054676680719</v>
       </c>
       <c r="BA58" t="n">
-        <v>5.528408572483942</v>
+        <v>0</v>
       </c>
       <c r="BB58" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC58" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9560,15 +9384,12 @@
         <v>-1.131721301339614</v>
       </c>
       <c r="AZ59" t="n">
-        <v>0.1468960643433882</v>
+        <v>1.468960643433882</v>
       </c>
       <c r="BA59" t="n">
-        <v>6.080598725084783</v>
+        <v>1</v>
       </c>
       <c r="BB59" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC59" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9713,15 +9534,12 @@
         <v>-1.148906986345209</v>
       </c>
       <c r="AZ60" t="n">
-        <v>0.1640718941643498</v>
+        <v>1.640718941643499</v>
       </c>
       <c r="BA60" t="n">
-        <v>4.620440023861259</v>
+        <v>0</v>
       </c>
       <c r="BB60" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9866,15 +9684,12 @@
         <v>-0.9802187884414533</v>
       </c>
       <c r="AZ61" t="n">
-        <v>0.2324436326842925</v>
+        <v>2.324436326842925</v>
       </c>
       <c r="BA61" t="n">
-        <v>6.589693642640406</v>
+        <v>1</v>
       </c>
       <c r="BB61" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC61" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10019,15 +9834,12 @@
         <v>-1.059967417806882</v>
       </c>
       <c r="AZ62" t="n">
-        <v>0.2271852849396293</v>
+        <v>2.271852849396293</v>
       </c>
       <c r="BA62" t="n">
-        <v>8.1219991100984</v>
+        <v>1</v>
       </c>
       <c r="BB62" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC62" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10172,15 +9984,12 @@
         <v>-1.07072599241777</v>
       </c>
       <c r="AZ63" t="n">
-        <v>0.2097736888129386</v>
+        <v>2.097736888129386</v>
       </c>
       <c r="BA63" t="n">
-        <v>6.659317142649229</v>
+        <v>1</v>
       </c>
       <c r="BB63" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC63" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10325,15 +10134,12 @@
         <v>-1.07072599241777</v>
       </c>
       <c r="AZ64" t="n">
-        <v>0.2051731480905204</v>
+        <v>2.051731480905203</v>
       </c>
       <c r="BA64" t="n">
-        <v>6.720409857723063</v>
+        <v>1</v>
       </c>
       <c r="BB64" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC64" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10478,15 +10284,12 @@
         <v>-1.072717162486702</v>
       </c>
       <c r="AZ65" t="n">
-        <v>0.1711270057226029</v>
+        <v>1.71127005722603</v>
       </c>
       <c r="BA65" t="n">
-        <v>6.465141386759904</v>
+        <v>0</v>
       </c>
       <c r="BB65" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC65" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10631,15 +10434,12 @@
         <v>-1.186907968195777</v>
       </c>
       <c r="AZ66" t="n">
-        <v>0.1264668813853405</v>
+        <v>1.264668813853404</v>
       </c>
       <c r="BA66" t="n">
-        <v>5.917373389442116</v>
+        <v>0</v>
       </c>
       <c r="BB66" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10784,15 +10584,12 @@
         <v>-1.05716724908219</v>
       </c>
       <c r="AZ67" t="n">
-        <v>0.1735620252135451</v>
+        <v>1.735620252135451</v>
       </c>
       <c r="BA67" t="n">
-        <v>5.130229695978934</v>
+        <v>0</v>
       </c>
       <c r="BB67" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC67" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10937,15 +10734,12 @@
         <v>-1.062612342442872</v>
       </c>
       <c r="AZ68" t="n">
-        <v>0.1651892043876882</v>
+        <v>1.651892043876882</v>
       </c>
       <c r="BA68" t="n">
-        <v>4.61721716535054</v>
+        <v>0</v>
       </c>
       <c r="BB68" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC68" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11090,15 +10884,12 @@
         <v>-1.162202419950019</v>
       </c>
       <c r="AZ69" t="n">
-        <v>0.1729739026459769</v>
+        <v>1.72973902645977</v>
       </c>
       <c r="BA69" t="n">
-        <v>4.169261023831525</v>
+        <v>0</v>
       </c>
       <c r="BB69" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC69" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11243,15 +11034,12 @@
         <v>-0.9735100220183867</v>
       </c>
       <c r="AZ70" t="n">
-        <v>0.1653302877966243</v>
+        <v>1.653302877966243</v>
       </c>
       <c r="BA70" t="n">
-        <v>5.468910140257988</v>
+        <v>0</v>
       </c>
       <c r="BB70" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC70" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11396,15 +11184,12 @@
         <v>-1.151540486656524</v>
       </c>
       <c r="AZ71" t="n">
-        <v>0.224534879706159</v>
+        <v>2.24534879706159</v>
       </c>
       <c r="BA71" t="n">
-        <v>6.385261085941602</v>
+        <v>0</v>
       </c>
       <c r="BB71" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC71" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11549,15 +11334,12 @@
         <v>-1.081507885923864</v>
       </c>
       <c r="AZ72" t="n">
-        <v>0.1704181532420173</v>
+        <v>1.704181532420173</v>
       </c>
       <c r="BA72" t="n">
-        <v>4.64552151410903</v>
+        <v>0</v>
       </c>
       <c r="BB72" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC72" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11702,15 +11484,12 @@
         <v>-1.008164398010397</v>
       </c>
       <c r="AZ73" t="n">
-        <v>0.1771344004138958</v>
+        <v>1.771344004138958</v>
       </c>
       <c r="BA73" t="n">
-        <v>5.317720031155273</v>
+        <v>0</v>
       </c>
       <c r="BB73" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC73" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11855,15 +11634,12 @@
         <v>-0.9019527661726316</v>
       </c>
       <c r="AZ74" t="n">
-        <v>0.2890653446677475</v>
+        <v>2.890653446677475</v>
       </c>
       <c r="BA74" t="n">
-        <v>7.650714677495467</v>
+        <v>0</v>
       </c>
       <c r="BB74" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC74" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12008,15 +11784,12 @@
         <v>-1.064321440481539</v>
       </c>
       <c r="AZ75" t="n">
-        <v>0.2678379030470969</v>
+        <v>2.678379030470969</v>
       </c>
       <c r="BA75" t="n">
-        <v>8.094394089102797</v>
+        <v>0</v>
       </c>
       <c r="BB75" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC75" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12161,15 +11934,12 @@
         <v>-1.036430349351861</v>
       </c>
       <c r="AZ76" t="n">
-        <v>0.2020516390549202</v>
+        <v>2.020516390549202</v>
       </c>
       <c r="BA76" t="n">
-        <v>6.613829372688381</v>
+        <v>0</v>
       </c>
       <c r="BB76" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC76" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12314,15 +12084,12 @@
         <v>-0.9447135609596995</v>
       </c>
       <c r="AZ77" t="n">
-        <v>0.2290004233178914</v>
+        <v>2.290004233178915</v>
       </c>
       <c r="BA77" t="n">
-        <v>6.379856596163442</v>
+        <v>0</v>
       </c>
       <c r="BB77" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC77" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12467,15 +12234,12 @@
         <v>-1.136069687512091</v>
       </c>
       <c r="AZ78" t="n">
-        <v>0.2143935207599353</v>
+        <v>2.143935207599353</v>
       </c>
       <c r="BA78" t="n">
-        <v>4.677253989798563</v>
+        <v>0</v>
       </c>
       <c r="BB78" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC78" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12620,15 +12384,12 @@
         <v>-0.7957323640055816</v>
       </c>
       <c r="AZ79" t="n">
-        <v>0.3250436485054538</v>
+        <v>3.250436485054538</v>
       </c>
       <c r="BA79" t="n">
-        <v>5.943353709831833</v>
+        <v>1</v>
       </c>
       <c r="BB79" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC79" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12773,15 +12534,12 @@
         <v>-1.083830924468203</v>
       </c>
       <c r="AZ80" t="n">
-        <v>0.2998648154876037</v>
+        <v>2.998648154876038</v>
       </c>
       <c r="BA80" t="n">
-        <v>6.635735356277657</v>
+        <v>1</v>
       </c>
       <c r="BB80" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC80" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12926,15 +12684,12 @@
         <v>-0.852490835998494</v>
       </c>
       <c r="AZ81" t="n">
-        <v>0.2994186256562353</v>
+        <v>2.994186256562354</v>
       </c>
       <c r="BA81" t="n">
-        <v>7.152431113667959</v>
+        <v>1</v>
       </c>
       <c r="BB81" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13079,15 +12834,12 @@
         <v>-1.073512489772441</v>
       </c>
       <c r="AZ82" t="n">
-        <v>0.1986099449474032</v>
+        <v>1.986099449474032</v>
       </c>
       <c r="BA82" t="n">
-        <v>5.80366638296212</v>
+        <v>1</v>
       </c>
       <c r="BB82" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC82" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13232,15 +12984,12 @@
         <v>-1.045162407612312</v>
       </c>
       <c r="AZ83" t="n">
-        <v>0.1574768288150041</v>
+        <v>1.574768288150041</v>
       </c>
       <c r="BA83" t="n">
-        <v>4.144199615258708</v>
+        <v>1</v>
       </c>
       <c r="BB83" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC83" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13385,15 +13134,12 @@
         <v>-1.011763599487811</v>
       </c>
       <c r="AZ84" t="n">
-        <v>0.1625698637855855</v>
+        <v>1.625698637855855</v>
       </c>
       <c r="BA84" t="n">
-        <v>4.910286937521602</v>
+        <v>1</v>
       </c>
       <c r="BB84" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC84" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13538,15 +13284,12 @@
         <v>-1.056436243301099</v>
       </c>
       <c r="AZ85" t="n">
-        <v>0.2261410104794487</v>
+        <v>2.261410104794487</v>
       </c>
       <c r="BA85" t="n">
-        <v>6.328175428570905</v>
+        <v>1</v>
       </c>
       <c r="BB85" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13691,15 +13434,12 @@
         <v>-1.139184969499528</v>
       </c>
       <c r="AZ86" t="n">
-        <v>0.2131678007547578</v>
+        <v>2.131678007547578</v>
       </c>
       <c r="BA86" t="n">
-        <v>6.522638295327906</v>
+        <v>1</v>
       </c>
       <c r="BB86" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC86" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13844,15 +13584,12 @@
         <v>-0.9994064701242487</v>
       </c>
       <c r="AZ87" t="n">
-        <v>0.2723142473493239</v>
+        <v>2.723142473493239</v>
       </c>
       <c r="BA87" t="n">
-        <v>7.354363492686352</v>
+        <v>1</v>
       </c>
       <c r="BB87" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC87" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13997,15 +13734,12 @@
         <v>-0.9530514877786842</v>
       </c>
       <c r="AZ88" t="n">
-        <v>0.2165437559626953</v>
+        <v>2.165437559626953</v>
       </c>
       <c r="BA88" t="n">
-        <v>4.352489670002637</v>
+        <v>1</v>
       </c>
       <c r="BB88" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC88" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14170,15 +13904,12 @@
         <v>-0.921325744894543</v>
       </c>
       <c r="AZ89" t="n">
-        <v>0.2273110803333757</v>
+        <v>2.273110803333757</v>
       </c>
       <c r="BA89" t="n">
-        <v>13.49936057389324</v>
+        <v>0</v>
       </c>
       <c r="BB89" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC89" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14343,15 +14074,12 @@
         <v>-0.9396264176117411</v>
       </c>
       <c r="AZ90" t="n">
-        <v>0.2562349769016561</v>
+        <v>2.562349769016562</v>
       </c>
       <c r="BA90" t="n">
-        <v>14.11226797838226</v>
+        <v>0</v>
       </c>
       <c r="BB90" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC90" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14516,15 +14244,12 @@
         <v>-0.9000000000000001</v>
       </c>
       <c r="AZ91" t="n">
-        <v>0.2747689268163115</v>
+        <v>2.747689268163116</v>
       </c>
       <c r="BA91" t="n">
-        <v>12.41339472150039</v>
+        <v>0</v>
       </c>
       <c r="BB91" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC91" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14689,15 +14414,12 @@
         <v>-0.9772876892692561</v>
       </c>
       <c r="AZ92" t="n">
-        <v>0.2638257036105743</v>
+        <v>2.638257036105744</v>
       </c>
       <c r="BA92" t="n">
-        <v>11.44644073918296</v>
+        <v>0</v>
       </c>
       <c r="BB92" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC92" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14862,15 +14584,12 @@
         <v>-0.8726919339164237</v>
       </c>
       <c r="AZ93" t="n">
-        <v>0.2205905999210828</v>
+        <v>2.205905999210828</v>
       </c>
       <c r="BA93" t="n">
-        <v>13.46108772447198</v>
+        <v>0</v>
       </c>
       <c r="BB93" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC93" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15035,15 +14754,12 @@
         <v>-0.8030209617755858</v>
       </c>
       <c r="AZ94" t="n">
-        <v>0.2899244513121407</v>
+        <v>2.899244513121407</v>
       </c>
       <c r="BA94" t="n">
-        <v>14.55098595795598</v>
+        <v>1</v>
       </c>
       <c r="BB94" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15208,15 +14924,12 @@
         <v>-0.9410150891632374</v>
       </c>
       <c r="AZ95" t="n">
-        <v>0.3639814907180162</v>
+        <v>3.639814907180162</v>
       </c>
       <c r="BA95" t="n">
-        <v>16.21005166131244</v>
+        <v>0</v>
       </c>
       <c r="BB95" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC95" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15381,15 +15094,12 @@
         <v>-0.8697027197975964</v>
       </c>
       <c r="AZ96" t="n">
-        <v>0.2754165199655664</v>
+        <v>2.754165199655663</v>
       </c>
       <c r="BA96" t="n">
-        <v>11.5432612977339</v>
+        <v>1</v>
       </c>
       <c r="BB96" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC96" t="n">
         <v>1</v>
       </c>
     </row>
@@ -15554,15 +15264,12 @@
         <v>-0.8926196808510639</v>
       </c>
       <c r="AZ97" t="n">
-        <v>0.2635851161810385</v>
+        <v>2.635851161810386</v>
       </c>
       <c r="BA97" t="n">
-        <v>18.63708247181081</v>
+        <v>0</v>
       </c>
       <c r="BB97" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC97" t="n">
         <v>1</v>
       </c>
     </row>
@@ -15727,15 +15434,12 @@
         <v>-0.9120214909335124</v>
       </c>
       <c r="AZ98" t="n">
-        <v>0.2379812101557392</v>
+        <v>2.379812101557392</v>
       </c>
       <c r="BA98" t="n">
-        <v>13.36431271950471</v>
+        <v>0</v>
       </c>
       <c r="BB98" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC98" t="n">
         <v>1</v>
       </c>
     </row>
@@ -15900,15 +15604,12 @@
         <v>-0.9579330904272938</v>
       </c>
       <c r="AZ99" t="n">
-        <v>0.1937192235493845</v>
+        <v>1.937192235493844</v>
       </c>
       <c r="BA99" t="n">
-        <v>10.8080729022015</v>
+        <v>0</v>
       </c>
       <c r="BB99" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC99" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16073,15 +15774,12 @@
         <v>-0.8845169545745361</v>
       </c>
       <c r="AZ100" t="n">
-        <v>0.1937567807703534</v>
+        <v>1.937567807703533</v>
       </c>
       <c r="BA100" t="n">
-        <v>12.77530493515518</v>
+        <v>0</v>
       </c>
       <c r="BB100" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC100" t="n">
         <v>1</v>
       </c>
     </row>
@@ -16246,15 +15944,12 @@
         <v>-0.8345370978332239</v>
       </c>
       <c r="AZ101" t="n">
-        <v>0.2390186769233919</v>
+        <v>2.390186769233919</v>
       </c>
       <c r="BA101" t="n">
-        <v>14.95225993840202</v>
+        <v>0</v>
       </c>
       <c r="BB101" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC101" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16419,15 +16114,12 @@
         <v>-0.8655913978494624</v>
       </c>
       <c r="AZ102" t="n">
-        <v>0.3022826134073608</v>
+        <v>3.022826134073608</v>
       </c>
       <c r="BA102" t="n">
-        <v>14.56543934132861</v>
+        <v>1</v>
       </c>
       <c r="BB102" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC102" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16592,15 +16284,12 @@
         <v>-0.8713188220230473</v>
       </c>
       <c r="AZ103" t="n">
-        <v>0.2697981424651091</v>
+        <v>2.697981424651091</v>
       </c>
       <c r="BA103" t="n">
-        <v>13.085308400592</v>
+        <v>1</v>
       </c>
       <c r="BB103" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC103" t="n">
         <v>1</v>
       </c>
     </row>
@@ -16765,15 +16454,12 @@
         <v>-0.873405299313052</v>
       </c>
       <c r="AZ104" t="n">
-        <v>0.3273385634947573</v>
+        <v>3.273385634947574</v>
       </c>
       <c r="BA104" t="n">
-        <v>13.77626263997392</v>
+        <v>1</v>
       </c>
       <c r="BB104" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC104" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16938,15 +16624,12 @@
         <v>-0.7809629835791817</v>
       </c>
       <c r="AZ105" t="n">
-        <v>0.2627407067212578</v>
+        <v>2.627407067212578</v>
       </c>
       <c r="BA105" t="n">
-        <v>13.64813509985642</v>
+        <v>1</v>
       </c>
       <c r="BB105" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC105" t="n">
         <v>0</v>
       </c>
     </row>
@@ -17111,15 +16794,12 @@
         <v>-0.9106683804627249</v>
       </c>
       <c r="AZ106" t="n">
-        <v>0.2253565398386968</v>
+        <v>2.253565398386967</v>
       </c>
       <c r="BA106" t="n">
-        <v>12.53521760130511</v>
+        <v>0</v>
       </c>
       <c r="BB106" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC106" t="n">
         <v>1</v>
       </c>
     </row>
@@ -17284,15 +16964,12 @@
         <v>-0.840602950609365</v>
       </c>
       <c r="AZ107" t="n">
-        <v>0.2310070069738794</v>
+        <v>2.310070069738794</v>
       </c>
       <c r="BA107" t="n">
-        <v>13.61822728292262</v>
+        <v>0</v>
       </c>
       <c r="BB107" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -17457,15 +17134,12 @@
         <v>-0.9048231511254019</v>
       </c>
       <c r="AZ108" t="n">
-        <v>0.2004180823301927</v>
+        <v>2.004180823301927</v>
       </c>
       <c r="BA108" t="n">
-        <v>12.36377526016233</v>
+        <v>0</v>
       </c>
       <c r="BB108" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC108" t="n">
         <v>1</v>
       </c>
     </row>
@@ -17630,15 +17304,12 @@
         <v>-0.8401015228426396</v>
       </c>
       <c r="AZ109" t="n">
-        <v>0.3164054433208752</v>
+        <v>3.164054433208753</v>
       </c>
       <c r="BA109" t="n">
-        <v>13.4521818706214</v>
+        <v>1</v>
       </c>
       <c r="BB109" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC109" t="n">
         <v>1</v>
       </c>
     </row>
@@ -17803,15 +17474,12 @@
         <v>-0.9122807017543859</v>
       </c>
       <c r="AZ110" t="n">
-        <v>0.3143298872640892</v>
+        <v>3.143298872640891</v>
       </c>
       <c r="BA110" t="n">
-        <v>13.71728615868613</v>
+        <v>0</v>
       </c>
       <c r="BB110" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC110" t="n">
         <v>0</v>
       </c>
     </row>
@@ -17976,15 +17644,12 @@
         <v>-0.9649181423321083</v>
       </c>
       <c r="AZ111" t="n">
-        <v>0.2727743536270423</v>
+        <v>2.727743536270423</v>
       </c>
       <c r="BA111" t="n">
-        <v>13.16711084989783</v>
+        <v>1</v>
       </c>
       <c r="BB111" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC111" t="n">
         <v>0</v>
       </c>
     </row>
@@ -18149,15 +17814,12 @@
         <v>-0.9372869802317655</v>
       </c>
       <c r="AZ112" t="n">
-        <v>0.2677287744794695</v>
+        <v>2.677287744794695</v>
       </c>
       <c r="BA112" t="n">
-        <v>14.90856583514423</v>
+        <v>0</v>
       </c>
       <c r="BB112" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC112" t="n">
         <v>1</v>
       </c>
     </row>
@@ -18322,15 +17984,12 @@
         <v>-0.8688741721854304</v>
       </c>
       <c r="AZ113" t="n">
-        <v>0.2699350840327465</v>
+        <v>2.699350840327465</v>
       </c>
       <c r="BA113" t="n">
-        <v>12.56625000971446</v>
+        <v>0</v>
       </c>
       <c r="BB113" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC113" t="n">
         <v>1</v>
       </c>
     </row>
@@ -18495,15 +18154,12 @@
         <v>-0.821639344262295</v>
       </c>
       <c r="AZ114" t="n">
-        <v>0.4709552277566549</v>
+        <v>4.70955227756655</v>
       </c>
       <c r="BA114" t="n">
-        <v>13.55543529737596</v>
+        <v>1</v>
       </c>
       <c r="BB114" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC114" t="n">
         <v>0</v>
       </c>
     </row>
@@ -18668,15 +18324,12 @@
         <v>-1.043353636689359</v>
       </c>
       <c r="AZ115" t="n">
-        <v>0.3439129986152255</v>
+        <v>3.439129986152254</v>
       </c>
       <c r="BA115" t="n">
-        <v>13.8462674929608</v>
+        <v>0</v>
       </c>
       <c r="BB115" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC115" t="n">
         <v>1</v>
       </c>
     </row>
@@ -18841,15 +18494,12 @@
         <v>-1.023550087873462</v>
       </c>
       <c r="AZ116" t="n">
-        <v>0.3494573532195661</v>
+        <v>3.494573532195661</v>
       </c>
       <c r="BA116" t="n">
-        <v>14.06948853210919</v>
+        <v>0</v>
       </c>
       <c r="BB116" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC116" t="n">
         <v>1</v>
       </c>
     </row>
@@ -19014,15 +18664,12 @@
         <v>-0.9992862241256246</v>
       </c>
       <c r="AZ117" t="n">
-        <v>0.2941786834792475</v>
+        <v>2.941786834792475</v>
       </c>
       <c r="BA117" t="n">
-        <v>11.36362404621276</v>
+        <v>0</v>
       </c>
       <c r="BB117" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC117" t="n">
         <v>0</v>
       </c>
     </row>
@@ -19187,15 +18834,12 @@
         <v>-0.9220733427362482</v>
       </c>
       <c r="AZ118" t="n">
-        <v>0.2356234081045346</v>
+        <v>2.356234081045346</v>
       </c>
       <c r="BA118" t="n">
-        <v>11.21671934408004</v>
+        <v>0</v>
       </c>
       <c r="BB118" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC118" t="n">
         <v>1</v>
       </c>
     </row>
@@ -19360,15 +19004,12 @@
         <v>-0.9540313754104341</v>
       </c>
       <c r="AZ119" t="n">
-        <v>0.2664652002443708</v>
+        <v>2.664652002443708</v>
       </c>
       <c r="BA119" t="n">
-        <v>12.68492545010291</v>
+        <v>0</v>
       </c>
       <c r="BB119" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC119" t="n">
         <v>1</v>
       </c>
     </row>
@@ -19533,15 +19174,12 @@
         <v>-0.8568159529257928</v>
       </c>
       <c r="AZ120" t="n">
-        <v>0.4458705469717965</v>
+        <v>4.458705469717965</v>
       </c>
       <c r="BA120" t="n">
-        <v>16.98593273105596</v>
+        <v>1</v>
       </c>
       <c r="BB120" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -19706,15 +19344,12 @@
         <v>-0.8646491519787163</v>
       </c>
       <c r="AZ121" t="n">
-        <v>0.4809162989997219</v>
+        <v>4.809162989997219</v>
       </c>
       <c r="BA121" t="n">
-        <v>17.24069091284437</v>
+        <v>0</v>
       </c>
       <c r="BB121" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC121" t="n">
         <v>1</v>
       </c>
     </row>
@@ -19879,15 +19514,12 @@
         <v>-0.8040981061782054</v>
       </c>
       <c r="AZ122" t="n">
-        <v>0.2754411937467637</v>
+        <v>2.754411937467637</v>
       </c>
       <c r="BA122" t="n">
-        <v>12.9142850910087</v>
+        <v>0</v>
       </c>
       <c r="BB122" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC122" t="n">
         <v>1</v>
       </c>
     </row>
@@ -20052,15 +19684,12 @@
         <v>-0.9652323580034423</v>
       </c>
       <c r="AZ123" t="n">
-        <v>0.2712645733328085</v>
+        <v>2.712645733328085</v>
       </c>
       <c r="BA123" t="n">
-        <v>13.89093963768983</v>
+        <v>0</v>
       </c>
       <c r="BB123" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC123" t="n">
         <v>1</v>
       </c>
     </row>
@@ -20225,15 +19854,12 @@
         <v>-0.9461077844311376</v>
       </c>
       <c r="AZ124" t="n">
-        <v>0.3551411071187895</v>
+        <v>3.551411071187895</v>
       </c>
       <c r="BA124" t="n">
-        <v>15.89478030353562</v>
+        <v>1</v>
       </c>
       <c r="BB124" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC124" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20398,15 +20024,12 @@
         <v>-0.9985683607730851</v>
       </c>
       <c r="AZ125" t="n">
-        <v>0.307205325190028</v>
+        <v>3.07205325190028</v>
       </c>
       <c r="BA125" t="n">
-        <v>11.82301848502743</v>
+        <v>1</v>
       </c>
       <c r="BB125" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC125" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20571,15 +20194,12 @@
         <v>-0.8554932365555923</v>
       </c>
       <c r="AZ126" t="n">
-        <v>0.3403595277379776</v>
+        <v>3.403595277379776</v>
       </c>
       <c r="BA126" t="n">
-        <v>12.94346879140066</v>
+        <v>1</v>
       </c>
       <c r="BB126" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC126" t="n">
         <v>1</v>
       </c>
     </row>
@@ -20744,15 +20364,12 @@
         <v>-0.8341742347796839</v>
       </c>
       <c r="AZ127" t="n">
-        <v>0.3160063990834164</v>
+        <v>3.160063990834163</v>
       </c>
       <c r="BA127" t="n">
-        <v>13.49082394850428</v>
+        <v>1</v>
       </c>
       <c r="BB127" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC127" t="n">
         <v>1</v>
       </c>
     </row>
@@ -20917,15 +20534,12 @@
         <v>-0.8899897505978819</v>
       </c>
       <c r="AZ128" t="n">
-        <v>0.3483273407058165</v>
+        <v>3.483273407058165</v>
       </c>
       <c r="BA128" t="n">
-        <v>14.95178371289261</v>
+        <v>0</v>
       </c>
       <c r="BB128" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC128" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21090,15 +20704,12 @@
         <v>-0.9594183293878932</v>
       </c>
       <c r="AZ129" t="n">
-        <v>0.3335399262952408</v>
+        <v>3.335399262952408</v>
       </c>
       <c r="BA129" t="n">
-        <v>13.39656411771</v>
+        <v>1</v>
       </c>
       <c r="BB129" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC129" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21263,15 +20874,12 @@
         <v>-0.8095535435529191</v>
       </c>
       <c r="AZ130" t="n">
-        <v>0.2816077793273518</v>
+        <v>2.816077793273518</v>
       </c>
       <c r="BA130" t="n">
-        <v>15.24780589347843</v>
+        <v>1</v>
       </c>
       <c r="BB130" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC130" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21436,15 +21044,12 @@
         <v>-0.8061192631907587</v>
       </c>
       <c r="AZ131" t="n">
-        <v>0.2283823895902871</v>
+        <v>2.283823895902871</v>
       </c>
       <c r="BA131" t="n">
-        <v>12.36588830848125</v>
+        <v>1</v>
       </c>
       <c r="BB131" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC131" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21609,15 +21214,12 @@
         <v>-0.9432647644326476</v>
       </c>
       <c r="AZ132" t="n">
-        <v>0.4425021074703185</v>
+        <v>4.425021074703185</v>
       </c>
       <c r="BA132" t="n">
-        <v>15.32398352756091</v>
+        <v>1</v>
       </c>
       <c r="BB132" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC132" t="n">
         <v>1</v>
       </c>
     </row>
@@ -21782,15 +21384,12 @@
         <v>-0.9047947568126941</v>
       </c>
       <c r="AZ133" t="n">
-        <v>0.3424239972728017</v>
+        <v>3.424239972728016</v>
       </c>
       <c r="BA133" t="n">
-        <v>15.37482698512445</v>
+        <v>0</v>
       </c>
       <c r="BB133" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC133" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21955,15 +21554,12 @@
         <v>-0.925575101488498</v>
       </c>
       <c r="AZ134" t="n">
-        <v>0.2877727947098655</v>
+        <v>2.877727947098654</v>
       </c>
       <c r="BA134" t="n">
-        <v>12.64306724710941</v>
+        <v>0</v>
       </c>
       <c r="BB134" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC134" t="n">
         <v>1</v>
       </c>
     </row>
@@ -22128,15 +21724,12 @@
         <v>-0.8729547641963427</v>
       </c>
       <c r="AZ135" t="n">
-        <v>0.2286543990281047</v>
+        <v>2.286543990281047</v>
       </c>
       <c r="BA135" t="n">
-        <v>14.34571921902312</v>
+        <v>0</v>
       </c>
       <c r="BB135" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC135" t="n">
         <v>1</v>
       </c>
     </row>
@@ -22301,15 +21894,12 @@
         <v>-0.8111718275652702</v>
       </c>
       <c r="AZ136" t="n">
-        <v>0.212522899192218</v>
+        <v>2.12522899192218</v>
       </c>
       <c r="BA136" t="n">
-        <v>12.07681251870081</v>
+        <v>0</v>
       </c>
       <c r="BB136" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC136" t="n">
         <v>1</v>
       </c>
     </row>
@@ -22474,15 +22064,12 @@
         <v>-0.9191253037139883</v>
       </c>
       <c r="AZ137" t="n">
-        <v>0.2487492359828174</v>
+        <v>2.487492359828174</v>
       </c>
       <c r="BA137" t="n">
-        <v>12.92788698041661</v>
+        <v>0</v>
       </c>
       <c r="BB137" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC137" t="n">
         <v>1</v>
       </c>
     </row>
@@ -22647,15 +22234,12 @@
         <v>-0.983991462113127</v>
       </c>
       <c r="AZ138" t="n">
-        <v>0.3634267201648407</v>
+        <v>3.634267201648408</v>
       </c>
       <c r="BA138" t="n">
-        <v>12.61555674855043</v>
+        <v>1</v>
       </c>
       <c r="BB138" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC138" t="n">
         <v>1</v>
       </c>
     </row>
@@ -22820,15 +22404,12 @@
         <v>-0.8676616915422886</v>
       </c>
       <c r="AZ139" t="n">
-        <v>0.3529111782529205</v>
+        <v>3.529111782529205</v>
       </c>
       <c r="BA139" t="n">
-        <v>14.94309852934265</v>
+        <v>0</v>
       </c>
       <c r="BB139" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC139" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22993,15 +22574,12 @@
         <v>-0.9794520547945206</v>
       </c>
       <c r="AZ140" t="n">
-        <v>0.2763025421902743</v>
+        <v>2.763025421902743</v>
       </c>
       <c r="BA140" t="n">
-        <v>13.50197279742473</v>
+        <v>1</v>
       </c>
       <c r="BB140" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC140" t="n">
         <v>1</v>
       </c>
     </row>
@@ -23166,15 +22744,12 @@
         <v>-0.8755935422602089</v>
       </c>
       <c r="AZ141" t="n">
-        <v>0.3071371534917146</v>
+        <v>3.071371534917147</v>
       </c>
       <c r="BA141" t="n">
-        <v>14.89304857028718</v>
+        <v>0</v>
       </c>
       <c r="BB141" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC141" t="n">
         <v>0</v>
       </c>
     </row>
@@ -23339,15 +22914,12 @@
         <v>-0.8558154437680231</v>
       </c>
       <c r="AZ142" t="n">
-        <v>0.2351665444744986</v>
+        <v>2.351665444744986</v>
       </c>
       <c r="BA142" t="n">
-        <v>12.33569292798704</v>
+        <v>0</v>
       </c>
       <c r="BB142" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC142" t="n">
         <v>0</v>
       </c>
     </row>
@@ -23512,15 +23084,12 @@
         <v>-0.910299003322259</v>
       </c>
       <c r="AZ143" t="n">
-        <v>0.2634069568539765</v>
+        <v>2.634069568539765</v>
       </c>
       <c r="BA143" t="n">
-        <v>13.20241292636161</v>
+        <v>0</v>
       </c>
       <c r="BB143" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC143" t="n">
         <v>0</v>
       </c>
     </row>
@@ -23685,15 +23254,12 @@
         <v>-0.8479307025986524</v>
       </c>
       <c r="AZ144" t="n">
-        <v>0.2850083474322018</v>
+        <v>2.850083474322018</v>
       </c>
       <c r="BA144" t="n">
-        <v>14.72041205661443</v>
+        <v>1</v>
       </c>
       <c r="BB144" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC144" t="n">
         <v>1</v>
       </c>
     </row>
@@ -23858,15 +23424,12 @@
         <v>-0.9031939413895291</v>
       </c>
       <c r="AZ145" t="n">
-        <v>0.3306302943724049</v>
+        <v>3.306302943724048</v>
       </c>
       <c r="BA145" t="n">
-        <v>13.50483650630982</v>
+        <v>1</v>
       </c>
       <c r="BB145" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC145" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24031,15 +23594,12 @@
         <v>-0.8867924528301887</v>
       </c>
       <c r="AZ146" t="n">
-        <v>0.3753925003975221</v>
+        <v>3.753925003975221</v>
       </c>
       <c r="BA146" t="n">
-        <v>14.04704424717668</v>
+        <v>0</v>
       </c>
       <c r="BB146" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC146" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24204,15 +23764,12 @@
         <v>-0.9927797833935018</v>
       </c>
       <c r="AZ147" t="n">
-        <v>0.275498874631122</v>
+        <v>2.754988746311219</v>
       </c>
       <c r="BA147" t="n">
-        <v>12.39357609552841</v>
+        <v>0</v>
       </c>
       <c r="BB147" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC147" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24377,15 +23934,12 @@
         <v>-0.8752424046541692</v>
       </c>
       <c r="AZ148" t="n">
-        <v>0.204352754630459</v>
+        <v>2.043527546304591</v>
       </c>
       <c r="BA148" t="n">
-        <v>12.73705359648974</v>
+        <v>0</v>
       </c>
       <c r="BB148" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC148" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24550,15 +24104,12 @@
         <v>-0.9457209457209457</v>
       </c>
       <c r="AZ149" t="n">
-        <v>0.1613708822578354</v>
+        <v>1.613708822578354</v>
       </c>
       <c r="BA149" t="n">
-        <v>10.17299216629021</v>
+        <v>0</v>
       </c>
       <c r="BB149" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC149" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24723,15 +24274,12 @@
         <v>-0.8900032351989647</v>
       </c>
       <c r="AZ150" t="n">
-        <v>0.2776338886342699</v>
+        <v>2.776338886342698</v>
       </c>
       <c r="BA150" t="n">
-        <v>15.42719268663395</v>
+        <v>0</v>
       </c>
       <c r="BB150" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC150" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24896,15 +24444,12 @@
         <v>-0.9144542772861356</v>
       </c>
       <c r="AZ151" t="n">
-        <v>0.1992943083149607</v>
+        <v>1.992943083149608</v>
       </c>
       <c r="BA151" t="n">
-        <v>12.29805279278685</v>
+        <v>0</v>
       </c>
       <c r="BB151" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC151" t="n">
         <v>0</v>
       </c>
     </row>
@@ -25069,15 +24614,12 @@
         <v>-0.870988867059594</v>
       </c>
       <c r="AZ152" t="n">
-        <v>0.2929222953305048</v>
+        <v>2.929222953305048</v>
       </c>
       <c r="BA152" t="n">
-        <v>13.84738554555246</v>
+        <v>1</v>
       </c>
       <c r="BB152" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC152" t="n">
         <v>0</v>
       </c>
     </row>
@@ -25242,15 +24784,12 @@
         <v>-0.9734422880490295</v>
       </c>
       <c r="AZ153" t="n">
-        <v>0.278928268195533</v>
+        <v>2.78928268195533</v>
       </c>
       <c r="BA153" t="n">
-        <v>12.99811599897735</v>
+        <v>1</v>
       </c>
       <c r="BB153" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC153" t="n">
         <v>1</v>
       </c>
     </row>
@@ -25415,15 +24954,12 @@
         <v>-0.8216748768472907</v>
       </c>
       <c r="AZ154" t="n">
-        <v>0.3594130595075935</v>
+        <v>3.594130595075935</v>
       </c>
       <c r="BA154" t="n">
-        <v>13.08294443919041</v>
+        <v>0</v>
       </c>
       <c r="BB154" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC154" t="n">
         <v>1</v>
       </c>
     </row>
@@ -25588,15 +25124,12 @@
         <v>-0.8612735542560104</v>
       </c>
       <c r="AZ155" t="n">
-        <v>0.2320891755316213</v>
+        <v>2.320891755316213</v>
       </c>
       <c r="BA155" t="n">
-        <v>12.9060602060763</v>
+        <v>0</v>
       </c>
       <c r="BB155" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC155" t="n">
         <v>0</v>
       </c>
     </row>
@@ -25761,15 +25294,12 @@
         <v>-1.018099547511312</v>
       </c>
       <c r="AZ156" t="n">
-        <v>0.3462797777914783</v>
+        <v>3.462797777914784</v>
       </c>
       <c r="BA156" t="n">
-        <v>14.93215294918606</v>
+        <v>0</v>
       </c>
       <c r="BB156" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC156" t="n">
         <v>1</v>
       </c>
     </row>
@@ -25934,15 +25464,12 @@
         <v>-1.04876299749014</v>
       </c>
       <c r="AZ157" t="n">
-        <v>0.3554401383644461</v>
+        <v>3.554401383644462</v>
       </c>
       <c r="BA157" t="n">
-        <v>15.32716274738345</v>
+        <v>0</v>
       </c>
       <c r="BB157" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC157" t="n">
         <v>1</v>
       </c>
     </row>
@@ -26107,15 +25634,12 @@
         <v>-0.8695652173913042</v>
       </c>
       <c r="AZ158" t="n">
-        <v>0.3274162961093018</v>
+        <v>3.274162961093018</v>
       </c>
       <c r="BA158" t="n">
-        <v>13.30667483923764</v>
+        <v>1</v>
       </c>
       <c r="BB158" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC158" t="n">
         <v>0</v>
       </c>
     </row>
@@ -26276,15 +25800,12 @@
       </c>
       <c r="AY159" t="inlineStr"/>
       <c r="AZ159" t="n">
-        <v>0.3352256061133059</v>
+        <v>3.352256061133059</v>
       </c>
       <c r="BA159" t="n">
-        <v>13.36339572806621</v>
+        <v>1</v>
       </c>
       <c r="BB159" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC159" t="n">
         <v>0</v>
       </c>
     </row>
@@ -26445,15 +25966,12 @@
       </c>
       <c r="AY160" t="inlineStr"/>
       <c r="AZ160" t="n">
-        <v>0.2434472726667247</v>
+        <v>2.434472726667246</v>
       </c>
       <c r="BA160" t="n">
-        <v>12.29154143560339</v>
+        <v>1</v>
       </c>
       <c r="BB160" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC160" t="n">
         <v>1</v>
       </c>
     </row>
@@ -26618,15 +26136,12 @@
         <v>-0.9148648648648647</v>
       </c>
       <c r="AZ161" t="n">
-        <v>0.2193729066609965</v>
+        <v>2.193729066609965</v>
       </c>
       <c r="BA161" t="n">
-        <v>11.64590440849937</v>
+        <v>0</v>
       </c>
       <c r="BB161" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC161" t="n">
         <v>1</v>
       </c>
     </row>
@@ -26791,15 +26306,12 @@
         <v>-0.875</v>
       </c>
       <c r="AZ162" t="n">
-        <v>0.2693134402703707</v>
+        <v>2.693134402703707</v>
       </c>
       <c r="BA162" t="n">
-        <v>12.17300558723502</v>
+        <v>1</v>
       </c>
       <c r="BB162" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC162" t="n">
         <v>0</v>
       </c>
     </row>
@@ -26964,15 +26476,12 @@
         <v>-0.9019350606756315</v>
       </c>
       <c r="AZ163" t="n">
-        <v>0.2786500146224659</v>
+        <v>2.786500146224659</v>
       </c>
       <c r="BA163" t="n">
-        <v>13.42169439208957</v>
+        <v>1</v>
       </c>
       <c r="BB163" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC163" t="n">
         <v>1</v>
       </c>
     </row>
@@ -27137,15 +26646,12 @@
         <v>-0.8602257636122178</v>
       </c>
       <c r="AZ164" t="n">
-        <v>0.3302696303234725</v>
+        <v>3.302696303234725</v>
       </c>
       <c r="BA164" t="n">
-        <v>14.07419437917497</v>
+        <v>1</v>
       </c>
       <c r="BB164" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC164" t="n">
         <v>1</v>
       </c>
     </row>
@@ -27310,15 +26816,12 @@
         <v>-0.8340425531914893</v>
       </c>
       <c r="AZ165" t="n">
-        <v>0.3140509103601919</v>
+        <v>3.140509103601919</v>
       </c>
       <c r="BA165" t="n">
-        <v>13.33772096173453</v>
+        <v>0</v>
       </c>
       <c r="BB165" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC165" t="n">
         <v>1</v>
       </c>
     </row>
@@ -27483,15 +26986,12 @@
         <v>-0.9123961218836566</v>
       </c>
       <c r="AZ166" t="n">
-        <v>0.4419867263324095</v>
+        <v>4.419867263324095</v>
       </c>
       <c r="BA166" t="n">
-        <v>16.97539046167085</v>
+        <v>1</v>
       </c>
       <c r="BB166" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC166" t="n">
         <v>0</v>
       </c>
     </row>
@@ -27656,15 +27156,12 @@
         <v>-0.9287135278514589</v>
       </c>
       <c r="AZ167" t="n">
-        <v>0.2822534280040117</v>
+        <v>2.822534280040117</v>
       </c>
       <c r="BA167" t="n">
-        <v>11.65132875248652</v>
+        <v>1</v>
       </c>
       <c r="BB167" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC167" t="n">
         <v>0</v>
       </c>
     </row>
@@ -27829,15 +27326,12 @@
         <v>-0.794580970384373</v>
       </c>
       <c r="AZ168" t="n">
-        <v>0.3720589980627997</v>
+        <v>3.720589980627997</v>
       </c>
       <c r="BA168" t="n">
-        <v>15.11954301763624</v>
+        <v>0</v>
       </c>
       <c r="BB168" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC168" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28002,15 +27496,12 @@
         <v>-0.8666886109282422</v>
       </c>
       <c r="AZ169" t="n">
-        <v>0.3370510290002701</v>
+        <v>3.370510290002701</v>
       </c>
       <c r="BA169" t="n">
-        <v>12.83721020627359</v>
+        <v>0</v>
       </c>
       <c r="BB169" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC169" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28175,15 +27666,12 @@
         <v>-0.8734652114597544</v>
       </c>
       <c r="AZ170" t="n">
-        <v>0.3618600999053327</v>
+        <v>3.618600999053328</v>
       </c>
       <c r="BA170" t="n">
-        <v>15.67979022827618</v>
+        <v>0</v>
       </c>
       <c r="BB170" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC170" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28348,15 +27836,12 @@
         <v>-0.9163306451612903</v>
       </c>
       <c r="AZ171" t="n">
-        <v>0.254785183807967</v>
+        <v>2.547851838079669</v>
       </c>
       <c r="BA171" t="n">
-        <v>11.61765076524852</v>
+        <v>0</v>
       </c>
       <c r="BB171" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC171" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28521,15 +28006,12 @@
         <v>-0.8450749123366273</v>
       </c>
       <c r="AZ172" t="n">
-        <v>0.3188696860136649</v>
+        <v>3.18869686013665</v>
       </c>
       <c r="BA172" t="n">
-        <v>14.69626650381366</v>
+        <v>1</v>
       </c>
       <c r="BB172" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC172" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28694,15 +28176,12 @@
         <v>-0.8522613065326633</v>
       </c>
       <c r="AZ173" t="n">
-        <v>0.399707243754127</v>
+        <v>3.99707243754127</v>
       </c>
       <c r="BA173" t="n">
-        <v>12.47173871860493</v>
+        <v>1</v>
       </c>
       <c r="BB173" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC173" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28867,15 +28346,12 @@
         <v>-0.9190476190476191</v>
       </c>
       <c r="AZ174" t="n">
-        <v>0.3801718619146223</v>
+        <v>3.801718619146223</v>
       </c>
       <c r="BA174" t="n">
-        <v>14.2475185393632</v>
+        <v>0</v>
       </c>
       <c r="BB174" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC174" t="n">
         <v>0</v>
       </c>
     </row>
@@ -29040,15 +28516,12 @@
         <v>-0.8253346392425727</v>
       </c>
       <c r="AZ175" t="n">
-        <v>0.2470312536106503</v>
+        <v>2.470312536106503</v>
       </c>
       <c r="BA175" t="n">
-        <v>11.3388765448196</v>
+        <v>1</v>
       </c>
       <c r="BB175" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC175" t="n">
         <v>1</v>
       </c>
     </row>
@@ -29213,15 +28686,12 @@
         <v>-0.8593242365172189</v>
       </c>
       <c r="AZ176" t="n">
-        <v>0.2303895675632164</v>
+        <v>2.303895675632163</v>
       </c>
       <c r="BA176" t="n">
-        <v>10.92082410889718</v>
+        <v>1</v>
       </c>
       <c r="BB176" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC176" t="n">
         <v>1</v>
       </c>
     </row>
@@ -29386,15 +28856,12 @@
         <v>-1.011280931586608</v>
       </c>
       <c r="AZ177" t="n">
-        <v>0.2939442645614514</v>
+        <v>2.939442645614514</v>
       </c>
       <c r="BA177" t="n">
-        <v>13.1516753899925</v>
+        <v>1</v>
       </c>
       <c r="BB177" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC177" t="n">
         <v>1</v>
       </c>
     </row>
@@ -29559,15 +29026,12 @@
         <v>-0.8638230647709321</v>
       </c>
       <c r="AZ178" t="n">
-        <v>0.3054467120359153</v>
+        <v>3.054467120359153</v>
       </c>
       <c r="BA178" t="n">
-        <v>13.45013914035445</v>
+        <v>1</v>
       </c>
       <c r="BB178" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC178" t="n">
         <v>1</v>
       </c>
     </row>
@@ -29732,15 +29196,12 @@
         <v>-0.8194444444444445</v>
       </c>
       <c r="AZ179" t="n">
-        <v>0.2464363334952325</v>
+        <v>2.464363334952325</v>
       </c>
       <c r="BA179" t="n">
-        <v>13.35702874314139</v>
+        <v>1</v>
       </c>
       <c r="BB179" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC179" t="n">
         <v>0</v>
       </c>
     </row>
@@ -29905,15 +29366,12 @@
         <v>-0.8907371167645139</v>
       </c>
       <c r="AZ180" t="n">
-        <v>0.3280651598232026</v>
+        <v>3.280651598232026</v>
       </c>
       <c r="BA180" t="n">
-        <v>12.92183174935129</v>
+        <v>0</v>
       </c>
       <c r="BB180" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC180" t="n">
         <v>0</v>
       </c>
     </row>
@@ -30078,15 +29536,12 @@
         <v>-0.9359058207979072</v>
       </c>
       <c r="AZ181" t="n">
-        <v>0.3562090494563998</v>
+        <v>3.562090494563997</v>
       </c>
       <c r="BA181" t="n">
-        <v>15.23965851812918</v>
+        <v>1</v>
       </c>
       <c r="BB181" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC181" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>